<commit_message>
Daten-Sync und Audiozuordnung vereinheitlichen
</commit_message>
<xml_diff>
--- a/wortliste/Tabelle.xlsx
+++ b/wortliste/Tabelle.xlsx
@@ -5397,7 +5397,7 @@
     <row r="345">
       <c r="B345" s="45" t="inlineStr">
         <is>
-          <t>Bass ( in Bass kurm)</t>
+          <t>Bass (in Bass kurm)</t>
         </is>
       </c>
       <c r="C345" s="45" t="inlineStr">
@@ -10739,7 +10739,7 @@
       </c>
       <c r="C711" s="45" t="inlineStr">
         <is>
-          <t>Hand- und Spanndienste (unent\-gelt\-lich für die Kommune )</t>
+          <t>Hand- und Spanndienste (unent\-gelt\-lich für die Kommune)</t>
         </is>
       </c>
     </row>
@@ -29941,7 +29941,7 @@
       </c>
       <c r="C2040" s="45" t="inlineStr">
         <is>
-          <t>aufklappen (Schuh), schlackern ( hat noch Luft)</t>
+          <t>aufklappen (Schuh), schlackern (hat noch Luft)</t>
         </is>
       </c>
     </row>
@@ -83470,7 +83470,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="23.25" customHeight="1" s="41">
       <c r="A30" s="38" t="inlineStr">
         <is>
@@ -85648,7 +85647,7 @@
       </c>
       <c r="B171" s="45" t="inlineStr">
         <is>
-          <t>Eigenwillige Kinder bekommen Schläge mit der Zwille (Stock) .</t>
+          <t>Eigenwillige Kinder bekommen Schläge mit der Zwille (Stock).</t>
         </is>
       </c>
     </row>
@@ -86357,7 +86356,6 @@
       <c r="B1" s="5" t="n"/>
       <c r="C1" s="5" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="17.4" customFormat="1" customHeight="1" s="4">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -86545,7 +86543,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="17.4" customFormat="1" customHeight="1" s="4">
       <c r="A40" s="4" t="inlineStr">
         <is>
@@ -86635,9 +86632,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -86694,9 +86688,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recorder-taugliche Schreibweise für Redewendungen
</commit_message>
<xml_diff>
--- a/wortliste/Tabelle.xlsx
+++ b/wortliste/Tabelle.xlsx
@@ -83570,7 +83570,7 @@
     <row r="2" ht="27.75" customHeight="1" s="41">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>"Meinemann" es daute, "Froagoars" lierbet nau.</t>
+          <t>„Meinemann“ es daute, „Froagoars“ lierbet nau.</t>
         </is>
       </c>
       <c r="B2" s="45" t="inlineStr">
@@ -83582,7 +83582,7 @@
     <row r="3" ht="27.75" customHeight="1" s="41">
       <c r="A3" s="45" t="inlineStr">
         <is>
-          <t>"Meinen", dat drügg, oaber wenn diu in de Böxen schiss, dat es gewiss.</t>
+          <t>„Meinen“, dat drügg, oaber wenn diu in de Böxen schiss, dat es gewiss.</t>
         </is>
       </c>
       <c r="B3" s="45" t="inlineStr">
@@ -84739,7 +84739,7 @@
     <row r="97" ht="27.75" customHeight="1" s="41">
       <c r="A97" s="45" t="inlineStr">
         <is>
-          <t>Et / Hei häf ein'n dürdraaihet.</t>
+          <t>Et ／ Hei häf ein'n dürdraaihet.</t>
         </is>
       </c>
       <c r="B97" s="45" t="inlineStr">
@@ -85096,7 +85096,7 @@
     <row r="126" ht="27" customHeight="1" s="41">
       <c r="A126" s="45" t="inlineStr">
         <is>
-          <t>Häff hei/et denn schon wat anhoalt?</t>
+          <t>Häff hei／et denn schon wat anhoalt?</t>
         </is>
       </c>
       <c r="B126" s="45" t="inlineStr">
@@ -85146,7 +85146,7 @@
     <row r="130" ht="27" customHeight="1" s="41">
       <c r="A130" s="45" t="inlineStr">
         <is>
-          <t>Hei / Et es geot inschloan.</t>
+          <t>Hei ／ Et es geot inschloan.</t>
         </is>
       </c>
       <c r="B130" s="45" t="inlineStr">
@@ -85558,7 +85558,7 @@
     <row r="164" ht="13.2" customHeight="1" s="41">
       <c r="A164" s="45" t="inlineStr">
         <is>
-          <t>Hei/et häff nix teoteosetten.</t>
+          <t>Hei／et häff nix teoteosetten.</t>
         </is>
       </c>
       <c r="B164" s="45" t="inlineStr">
@@ -86117,7 +86117,7 @@
     <row r="210" ht="13.2" customHeight="1" s="41">
       <c r="A210" s="45" t="inlineStr">
         <is>
-          <t>Wat sägg de Irsel, wenn hei in de Mührlen kummp? / Konns diu nich Doagestiet säggen?</t>
+          <t>Wat sägg de Irsel, wenn hei in de Mührlen kummp? ／ Konns diu nich Doagestiet säggen?</t>
         </is>
       </c>
       <c r="B210" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Schreibweisen für Alternativen und Auslassungen vereinheitlichen
</commit_message>
<xml_diff>
--- a/wortliste/Tabelle.xlsx
+++ b/wortliste/Tabelle.xlsx
@@ -12022,7 +12022,7 @@
 ich tue tat habe getan
 du tust tatest
 er, sie, es tut tat
-wir tun ... taten ...</t>
+wir tun … taten …</t>
         </is>
       </c>
     </row>
@@ -21517,7 +21517,7 @@
 ich glaube glaubte
 du glaubst glaubtest
 er, sie, es glaubt glaubte
-wir glauben ... glaubten</t>
+wir glauben … glaubten</t>
         </is>
       </c>
     </row>
@@ -21810,7 +21810,7 @@
 ich gehe ging bin gegangen
 du gehst gingst
 er, sie, es geht ging
-wir gehen ... gingen ...</t>
+wir gehen … gingen …</t>
         </is>
       </c>
     </row>
@@ -23466,7 +23466,7 @@
 ich habe hatte habe gehabt
 du hast hattest
 er, sie, es hat hatte
-wir haben ... hatten ...</t>
+wir haben … hatten …</t>
         </is>
       </c>
     </row>
@@ -23994,7 +23994,7 @@
 ich heiße hieß habe geheißen
 du heißt hießest
 er, sie, es heißt hieß
-wir heißen ... hießen ...</t>
+wir heißen … hießen …</t>
         </is>
       </c>
     </row>
@@ -26062,7 +26062,7 @@
 ich hoffe hoffte habe gehofft
 du hoffst hofftest
 er, sie, es hofft hoffte
-wir hoffen ... hofften ...</t>
+wir hoffen … hofften …</t>
         </is>
       </c>
     </row>
@@ -34743,7 +34743,7 @@
 ich kann konnte habe gekonnt
 du kannst konntest
 er, sie, es kann konnte
-wir können ... konnten ...</t>
+wir können … konnten …</t>
         </is>
       </c>
     </row>
@@ -35469,7 +35469,7 @@
 ich laufe lief bin gelaufen
 du läufst liefest
 er, sie, es läuft lief
-wir laufen ... liefen ...</t>
+wir laufen … liefen …</t>
         </is>
       </c>
     </row>
@@ -40211,7 +40211,7 @@
 ich muss musste habe gemusst
 du musst musstest
 er, sie, es muss musste
-wir müssen ... mussten ...</t>
+wir müssen … mussten …</t>
         </is>
       </c>
     </row>
@@ -51268,7 +51268,7 @@
       </c>
       <c r="C3464" s="45" t="inlineStr">
         <is>
-          <t>Maßeinheit (ein Sack voll ...)</t>
+          <t>Maßeinheit (ein Sack voll …)</t>
         </is>
       </c>
     </row>
@@ -51667,7 +51667,7 @@
 ich soll sollte habe gesollt
 du sollst solltest
 er, sie, es soll sollte
-wir sollen ... sollten ...</t>
+wir sollen … sollten …</t>
         </is>
       </c>
     </row>
@@ -57041,7 +57041,7 @@
 ich sehe sah habe gesehen
 du siehst sahst
 er, sie, es sieht sah
-wir sehen ... sahen ...</t>
+wir sehen … sahen …</t>
         </is>
       </c>
     </row>
@@ -57444,7 +57444,7 @@
 ich bin war bin gewesen
 du bist warst
 er, sie, es ist war
-wir sind ... waren ...</t>
+wir sind … waren …</t>
         </is>
       </c>
     </row>
@@ -77844,7 +77844,7 @@
 ich will wollte habe gewollt
 du willst wolltest
 er, sie, es will wollte
-wir wollen ... wollten ...</t>
+wir wollen … wollten …</t>
         </is>
       </c>
     </row>
@@ -84739,7 +84739,7 @@
     <row r="97" ht="27.75" customHeight="1" s="41">
       <c r="A97" s="45" t="inlineStr">
         <is>
-          <t>Et ／ Hei häf ein'n dürdraaihet.</t>
+          <t>Et／hei häf ein'n dürdraaihet.</t>
         </is>
       </c>
       <c r="B97" s="45" t="inlineStr">
@@ -85146,7 +85146,7 @@
     <row r="130" ht="27" customHeight="1" s="41">
       <c r="A130" s="45" t="inlineStr">
         <is>
-          <t>Hei ／ Et es geot inschloan.</t>
+          <t>Hei／et es geot inschloan.</t>
         </is>
       </c>
       <c r="B130" s="45" t="inlineStr">
@@ -85683,7 +85683,7 @@
       </c>
       <c r="B174" s="45" t="inlineStr">
         <is>
-          <t>Ein Hund auf dem Hof hat es besser als ….</t>
+          <t>Ein Hund auf dem Hof hat es besser als …</t>
         </is>
       </c>
       <c r="C174" s="49" t="n"/>

</xml_diff>